<commit_message>
Adding map visualisation into dashboard
</commit_message>
<xml_diff>
--- a/KL_Attraction_Place.xlsx
+++ b/KL_Attraction_Place.xlsx
@@ -1214,152 +1214,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>National Art Gallery</t>
+          <t>Merdeka Square</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Saloma Bridge</t>
+          <t>National Monument</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>KLCC</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>KL Tower</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>National Monument</t>
+          <t>Chinatown</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>National Art Gallery</t>
+          <t>Merdeka Square</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>3.11</v>
+        <v>1.28</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>5.22</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>6.25</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Saloma Bridge</t>
+          <t>National Monument</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>3.11</v>
+        <v>1.28</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>4.3</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>KLCC</t>
+          <t>Chinatown</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3.51</v>
+        <v>2.53</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2.31</v>
+        <v>2.24</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>4.91</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>KL Tower</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>5.22</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>3.46</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>National Monument</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>